<commit_message>
docs: rename ke SIMKERMA, perbarui README (link repo/live, langkah deploy), samakan BASE_URL
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_MonitoringKerjasama.xlsx
+++ b/Template_Spreadsheet_MonitoringKerjasama.xlsx
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -62,14 +61,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -603,9 +603,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>2</v>
       </c>
@@ -677,9 +674,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
         <v>2</v>
       </c>
@@ -708,9 +702,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>2</v>
       </c>
@@ -782,9 +773,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>2</v>
       </c>
@@ -813,9 +801,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
         <v>2</v>
       </c>
@@ -887,9 +872,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>2</v>
       </c>
@@ -961,9 +943,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
         <v>2</v>
       </c>
@@ -992,9 +971,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>2</v>
       </c>
@@ -1023,9 +999,6 @@
           <t>Jawa Barat</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>2</v>
       </c>
@@ -1054,9 +1027,6 @@
           <t>DKI Jakarta</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>2</v>
       </c>
@@ -1085,9 +1055,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>2</v>
       </c>
@@ -1116,9 +1083,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>2</v>
       </c>
@@ -1147,9 +1111,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
         <v>2</v>
       </c>
@@ -1178,9 +1139,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>0</v>
       </c>
@@ -1209,9 +1167,6 @@
           <t>Manila, Filipina</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
         <v>0</v>
       </c>
@@ -1240,9 +1195,6 @@
           <t>Sumatera Selatan</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>0</v>
       </c>
@@ -1418,7 +1370,7 @@
           <t>K-0015</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="5" t="n">
         <v>45435.375</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -1483,10 +1435,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -1500,7 +1448,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1508,7 +1455,7 @@
           <t>K-0004</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="5" t="n">
         <v>44032.375</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -1573,14 +1520,11 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
           <t>K-0003</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -1594,7 +1538,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1602,7 +1545,7 @@
           <t>K-0033</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="5" t="n">
         <v>45635.375</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -1667,10 +1610,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -1684,7 +1623,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1692,7 +1630,7 @@
           <t>K-0044</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="5" t="n">
         <v>44914.375</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -1757,10 +1695,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -1774,7 +1708,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1782,7 +1715,7 @@
           <t>K-0006</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="5" t="n">
         <v>45716.375</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -1847,14 +1780,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
           <t>K-0003</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -1868,7 +1798,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1876,7 +1805,7 @@
           <t>K-0031</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="5" t="n">
         <v>45026.375</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -1941,10 +1870,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -1958,7 +1883,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1966,7 +1890,7 @@
           <t>K-0009</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>45768.375</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -2031,10 +1955,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -2048,7 +1968,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2056,7 +1975,7 @@
           <t>K-0043</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>44308.375</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -2121,10 +2040,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -2138,7 +2053,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2146,7 +2060,7 @@
           <t>K-0045</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="5" t="n">
         <v>45424.375</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -2211,14 +2125,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>K-0046</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
           <t>Habis</t>
@@ -2232,7 +2143,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2240,7 +2150,7 @@
           <t>K-0039</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="5" t="n">
         <v>44395.375</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -2305,10 +2215,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2322,7 +2228,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2330,7 +2235,7 @@
           <t>K-0042</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="5" t="n">
         <v>45859.375</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -2395,14 +2300,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>K-0041</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2416,7 +2318,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2424,7 +2325,7 @@
           <t>K-0036</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="5" t="n">
         <v>45132.375</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -2489,10 +2390,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2506,7 +2403,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2514,7 +2410,7 @@
           <t>K-0046</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="5" t="n">
         <v>45870.375</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -2579,10 +2475,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2596,7 +2488,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2604,7 +2495,7 @@
           <t>K-0041</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="5" t="n">
         <v>45158.375</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -2669,10 +2560,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2686,7 +2573,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2694,7 +2580,7 @@
           <t>K-0047</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="5" t="n">
         <v>45527.375</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -2759,14 +2645,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>K-0048</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2780,7 +2663,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2788,7 +2670,7 @@
           <t>K-0010</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="5" t="n">
         <v>45165.375</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -2853,14 +2735,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>K-0007</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2874,7 +2753,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2882,7 +2760,7 @@
           <t>K-0012</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="5" t="n">
         <v>45901.375</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -2947,10 +2825,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -2964,7 +2838,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2972,7 +2845,7 @@
           <t>K-0029</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="5" t="n">
         <v>45923.375</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -3037,10 +2910,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
@@ -3054,7 +2923,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3062,7 +2930,7 @@
           <t>K-0037</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="5" t="n">
         <v>45723.375</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -3127,14 +2995,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>K-0038</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
-      <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3148,7 +3013,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3156,7 +3020,7 @@
           <t>K-0002</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="5" t="n">
         <v>44665.375</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -3221,14 +3085,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
           <t>K-0003</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3242,7 +3103,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3250,7 +3110,7 @@
           <t>K-0024</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="5" t="n">
         <v>45454.375</v>
       </c>
       <c r="C22" t="inlineStr">
@@ -3315,10 +3175,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3332,7 +3188,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3340,7 +3195,7 @@
           <t>K-0032</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="5" t="n">
         <v>45458.375</v>
       </c>
       <c r="C23" t="inlineStr">
@@ -3405,10 +3260,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3422,7 +3273,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3430,7 +3280,7 @@
           <t>K-0011</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="5" t="n">
         <v>45847.375</v>
       </c>
       <c r="C24" t="inlineStr">
@@ -3495,10 +3345,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3512,7 +3358,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3520,7 +3365,7 @@
           <t>K-0025</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="5" t="n">
         <v>45691.375</v>
       </c>
       <c r="C25" t="inlineStr">
@@ -3585,10 +3430,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3602,7 +3443,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3610,7 +3450,7 @@
           <t>K-0027</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="5" t="n">
         <v>46064.375</v>
       </c>
       <c r="C26" t="inlineStr">
@@ -3675,14 +3515,11 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr">
         <is>
           <t>K-0028</t>
         </is>
       </c>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3696,7 +3533,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3704,7 +3540,7 @@
           <t>K-0014</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="5" t="n">
         <v>46108.375</v>
       </c>
       <c r="C27" t="inlineStr">
@@ -3769,14 +3605,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>K-0015</t>
         </is>
       </c>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3790,7 +3623,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3798,7 +3630,7 @@
           <t>K-0038</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="5" t="n">
         <v>45058.375</v>
       </c>
       <c r="C28" t="inlineStr">
@@ -3863,10 +3695,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3880,7 +3708,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3888,7 +3715,7 @@
           <t>K-0035</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="5" t="n">
         <v>46524.375</v>
       </c>
       <c r="C29" t="inlineStr">
@@ -3953,10 +3780,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -3970,7 +3793,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3978,7 +3800,7 @@
           <t>K-0005</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="5" t="n">
         <v>45805.375</v>
       </c>
       <c r="C30" t="inlineStr">
@@ -4043,10 +3865,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4060,7 +3878,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4068,7 +3885,7 @@
           <t>K-0023</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="5" t="n">
         <v>46553.375</v>
       </c>
       <c r="C31" t="inlineStr">
@@ -4133,10 +3950,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4150,7 +3963,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4158,7 +3970,7 @@
           <t>K-0019</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="5" t="n">
         <v>46659.375</v>
       </c>
       <c r="C32" t="inlineStr">
@@ -4223,14 +4035,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr">
         <is>
           <t>K-0020</t>
         </is>
       </c>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4244,7 +4053,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4252,7 +4060,7 @@
           <t>K-0022</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="5" t="n">
         <v>45216.375</v>
       </c>
       <c r="C33" t="inlineStr">
@@ -4317,10 +4125,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4334,7 +4138,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4342,7 +4145,7 @@
           <t>K-0021</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="5" t="n">
         <v>45978.375</v>
       </c>
       <c r="C34" t="inlineStr">
@@ -4407,10 +4210,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4424,7 +4223,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4432,7 +4230,7 @@
           <t>K-0040</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="5" t="n">
         <v>46364.375</v>
       </c>
       <c r="C35" t="inlineStr">
@@ -4497,10 +4295,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4514,7 +4308,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4522,7 +4315,7 @@
           <t>K-0003</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="5" t="n">
         <v>46000.375</v>
       </c>
       <c r="C36" t="inlineStr">
@@ -4587,10 +4380,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4604,7 +4393,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4612,7 +4400,7 @@
           <t>K-0017</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="5" t="n">
         <v>45286.375</v>
       </c>
       <c r="C37" t="inlineStr">
@@ -4677,10 +4465,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4694,7 +4478,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4702,7 +4485,7 @@
           <t>K-0008</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="5" t="n">
         <v>46070.375</v>
       </c>
       <c r="C38" t="inlineStr">
@@ -4767,14 +4550,11 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr">
         <is>
           <t>K-0007</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4788,7 +4568,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4796,7 +4575,7 @@
           <t>K-0016</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="5" t="n">
         <v>46119.375</v>
       </c>
       <c r="C39" t="inlineStr">
@@ -4861,10 +4640,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4878,7 +4653,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4886,7 +4660,7 @@
           <t>K-0026</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="5" t="n">
         <v>46549.375</v>
       </c>
       <c r="C40" t="inlineStr">
@@ -4951,10 +4725,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -4968,7 +4738,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4976,7 +4745,7 @@
           <t>K-0007</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="5" t="n">
         <v>45462.375</v>
       </c>
       <c r="C41" t="inlineStr">
@@ -5041,10 +4810,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5058,7 +4823,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5066,7 +4830,7 @@
           <t>K-0001</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="5" t="n">
         <v>46924.375</v>
       </c>
       <c r="C42" t="inlineStr">
@@ -5131,14 +4895,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr">
         <is>
           <t>K-0003</t>
         </is>
       </c>
-      <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5152,7 +4913,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5160,7 +4920,7 @@
           <t>K-0020</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="5" t="n">
         <v>46221.375</v>
       </c>
       <c r="C43" t="inlineStr">
@@ -5225,10 +4985,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5242,7 +4998,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5250,7 +5005,7 @@
           <t>K-0028</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="5" t="n">
         <v>46229.375</v>
       </c>
       <c r="C44" t="inlineStr">
@@ -5315,10 +5070,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
-      <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5332,7 +5083,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5340,7 +5090,7 @@
           <t>K-0048</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="5" t="n">
         <v>47048.375</v>
       </c>
       <c r="C45" t="inlineStr">
@@ -5405,10 +5155,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5422,7 +5168,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5430,7 +5175,7 @@
           <t>K-0030</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="5" t="n">
         <v>46323.375</v>
       </c>
       <c r="C46" t="inlineStr">
@@ -5495,14 +5240,11 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
           <t>K-0029</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr"/>
-      <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5516,7 +5258,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5524,7 +5265,7 @@
           <t>K-0034</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="5" t="n">
         <v>45606.375</v>
       </c>
       <c r="C47" t="inlineStr">
@@ -5589,10 +5330,6 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5606,7 +5343,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5614,7 +5350,7 @@
           <t>K-0013</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="5" t="n">
         <v>47088.375</v>
       </c>
       <c r="C48" t="inlineStr">
@@ -5679,14 +5415,11 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
       <c r="R48" t="inlineStr">
         <is>
           <t>K-0015</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr"/>
-      <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5700,7 +5433,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5708,7 +5440,7 @@
           <t>K-0018</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="5" t="n">
         <v>46387.375</v>
       </c>
       <c r="C49" t="inlineStr">
@@ -5773,10 +5505,6 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr">
         <is>
           <t>Aktif</t>
@@ -5790,7 +5518,6 @@
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6536,7 +6263,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://monitoring-kerjasama.vercel.app</t>
+          <t>https://simkerma.vercel.app</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -6602,7 +6329,6 @@
           <t>WA_TARGET</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Nomor WhatsApp tujuan (mis. 62812xxxx), pisahkan koma</t>

</xml_diff>

<commit_message>
refactor(survey): pindahkan toggle SURVEY_AKTIF ke tab Pengaturan (bukan env)
- SURVEY_AKTIF kini kunci Pengaturan (default TRUE) → on/off overlay survei
  tanpa redeploy. Endpoint publik getPublicConfig mengembalikan { surveyAktif }.
- app.js: overlay baca toggle via getPublicConfig, di-cache ~6 jam di localStorage
  (gagal ambil → overlay tidak tampil). Hapus konstanta env SURVEY_AKTIF.
- build.js & .env.example: buang SURVEY_AKTIF (URL form tetap env).
- Template + builder: tambah kunci SURVEY_AKTIF. Docs README disesuaikan.
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_MonitoringKerjasama.xlsx
+++ b/Template_Spreadsheet_MonitoringKerjasama.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mitra'!$A$1:$I$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kerjasama'!$A$1:$X$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dataset'!$A$1:$B$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pengaturan'!$A$1:$C$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pengaturan'!$A$1:$C$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -149,6 +149,12 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9333,7 +9339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9359,12 +9365,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>NAMA_INSTANSI</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Politeknik Kesehatan Kemenkes Palembang</t>
         </is>
@@ -9376,12 +9382,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>EMAIL_NOTIF</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -9393,12 +9399,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>BASE_URL</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>https://simkerma.vercel.app</t>
         </is>
@@ -9410,12 +9416,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>REMINDER_CADENCE</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>90:30,60:14,30:7,7:1</t>
         </is>
@@ -9427,12 +9433,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>GRACE_HABIS_HARI</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="14" t="n">
         <v>14</v>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -9442,12 +9448,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>EMAIL_AKTIF</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -9459,12 +9465,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>WA_NOMOR_AKTIF</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9476,12 +9482,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>WA_TARGET</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr"/>
+      <c r="B9" s="14" t="inlineStr"/>
       <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Nomor WA tim internal (mis. 62812xxxx), pisahkan koma</t>
@@ -9489,12 +9495,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>WA_GRUP_AKTIF</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9506,12 +9512,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>WA_GRUP_ID</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr"/>
+      <c r="B11" s="14" t="inlineStr"/>
       <c r="C11" s="12" t="inlineStr">
         <is>
           <t>ID grup WhatsApp (Fonnte) untuk rekap internal</t>
@@ -9519,12 +9525,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>LAMPIRKAN_FILE</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -9536,12 +9542,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>EMAIL_EKSTERNAL_AKTIF</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9553,12 +9559,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>WA_EKSTERNAL_AKTIF</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9570,12 +9576,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>WA_EKSTERNAL_MAKS_PER_HARI</t>
         </is>
       </c>
-      <c r="B15" s="11" t="n">
+      <c r="B15" s="14" t="n">
         <v>8</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -9585,12 +9591,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>WA_EKSTERNAL_JEDA_DETIK</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B16" s="14" t="n">
         <v>8</v>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -9599,8 +9605,25 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>SURVEY_AKTIF</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Tampilkan overlay survei tahunan (mulai November). FALSE = matikan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C16"/>
+  <autoFilter ref="A1:C17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(kerjasama): kolom Tindak Lanjut + stop-notif + auto-tutup perpanjangan
- Kolom baru 'Tindak Lanjut': kosong/'Sedang Diproses' = terus diingatkan;
  'Diperpanjang'/'Tidak Diperpanjang'/'Selesai' = pengingat berhenti (_tlClosed).
- cekDanKirimReminder & diagReminder menghormati Tindak Lanjut (skip yang ditutup).
- Perpanjangan: form kini memilih KERJA SAMA sebelumnya (bukan cuma mitra) via
  #refKerjasama (wajib) → refSebelumnya benar; backend auto-set baris lama 'Diperpanjang'
  (_tandaiDiperpanjang) sehingga notifnya berhenti. Perbaiki bug ref=id mitra.
- form.html/form.js: field Tindak Lanjut + 'Kerja Sama yang Diperpanjang' + prefill edit.
- data table: kolom Tindak Lanjut (badge) + di detail expand.
- Template + builder: kolom Tindak Lanjut + ~20 baris UJI notif (sebar semua zona cadence,
  termasuk 1 'Tidak Diperpanjang' utk uji stop). _listKerjasama & migrasi disesuaikan.
</commit_message>
<xml_diff>
--- a/Template_Spreadsheet_MonitoringKerjasama.xlsx
+++ b/Template_Spreadsheet_MonitoringKerjasama.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mitra'!$A$1:$I$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kerjasama'!$A$1:$X$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kerjasama'!$A$1:$Y$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dataset'!$A$1:$B$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pengaturan'!$A$1:$C$17</definedName>
   </definedNames>
@@ -24,9 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -126,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -150,6 +151,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1972,7 +1980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X76"/>
+  <dimension ref="A1:Y96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1995,10 +2003,11 @@
     <col width="26" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="24" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="24" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2104,20 +2113,25 @@
       </c>
       <c r="U1" s="6" t="inlineStr">
         <is>
+          <t>Tindak Lanjut</t>
+        </is>
+      </c>
+      <c r="V1" s="6" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="V1" s="6" t="inlineStr">
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>Sisa Hari</t>
         </is>
       </c>
-      <c r="W1" s="6" t="inlineStr">
+      <c r="X1" s="6" t="inlineStr">
         <is>
           <t>Diinput Oleh</t>
         </is>
       </c>
-      <c r="X1" s="6" t="inlineStr">
+      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>Reminder Terakhir</t>
         </is>
@@ -2199,15 +2213,15 @@
           <t>Riset bersama; konfirmasi lanjut</t>
         </is>
       </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="V2" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>19</v>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2284,15 +2298,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U3" s="7" t="inlineStr">
+      <c r="V3" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>29</v>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2379,15 +2393,15 @@
           <t>Segera jatuh tempo, siapkan perpanjangan</t>
         </is>
       </c>
-      <c r="U4" s="7" t="inlineStr">
+      <c r="V4" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>44</v>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2464,15 +2478,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U5" s="7" t="inlineStr">
+      <c r="V5" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>59</v>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2554,15 +2568,15 @@
           <t>Sudah diperpanjang</t>
         </is>
       </c>
-      <c r="U6" s="8" t="inlineStr">
+      <c r="V6" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>-470</v>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2644,15 +2658,15 @@
           <t>Habis baru-baru ini</t>
         </is>
       </c>
-      <c r="U7" s="8" t="inlineStr">
+      <c r="V7" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>-41</v>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2739,15 +2753,15 @@
           <t>Menunggu konfirmasi mitra untuk perpanjangan</t>
         </is>
       </c>
-      <c r="U8" s="8" t="inlineStr">
+      <c r="V8" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>-31</v>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2829,15 +2843,15 @@
           <t>Berakhir hari ini — segera tindak lanjut</t>
         </is>
       </c>
-      <c r="U9" s="8" t="inlineStr">
+      <c r="V9" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>-1</v>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -2919,15 +2933,15 @@
           <t>Kontrak penyediaan tenaga; nilai besar</t>
         </is>
       </c>
-      <c r="U10" s="9" t="inlineStr">
+      <c r="V10" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>164</v>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3004,15 +3018,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U11" s="9" t="inlineStr">
+      <c r="V11" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>164</v>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3094,15 +3108,15 @@
           <t>Tidak diperpanjang — klinik pindah kepemilikan</t>
         </is>
       </c>
-      <c r="U12" s="9" t="inlineStr">
+      <c r="V12" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>229</v>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3189,15 +3203,15 @@
           <t>Addendum penambahan ruang lingkup</t>
         </is>
       </c>
-      <c r="U13" s="9" t="inlineStr">
+      <c r="V13" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>344</v>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3274,15 +3288,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U14" s="9" t="inlineStr">
+      <c r="V14" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V14" t="n">
+      <c r="W14" t="n">
         <v>349</v>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3359,15 +3373,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U15" s="9" t="inlineStr">
+      <c r="V15" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V15" t="n">
+      <c r="W15" t="n">
         <v>429</v>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3444,15 +3458,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U16" s="9" t="inlineStr">
+      <c r="V16" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V16" t="n">
+      <c r="W16" t="n">
         <v>630</v>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3529,15 +3543,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U17" s="9" t="inlineStr">
+      <c r="V17" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V17" t="n">
+      <c r="W17" t="n">
         <v>710</v>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3614,15 +3628,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U18" s="9" t="inlineStr">
+      <c r="V18" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V18" t="n">
+      <c r="W18" t="n">
         <v>770</v>
       </c>
-      <c r="W18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3699,15 +3713,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U19" s="9" t="inlineStr">
+      <c r="V19" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V19" t="n">
+      <c r="W19" t="n">
         <v>800</v>
       </c>
-      <c r="W19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3784,15 +3798,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U20" s="9" t="inlineStr">
+      <c r="V20" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V20" t="n">
+      <c r="W20" t="n">
         <v>815</v>
       </c>
-      <c r="W20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3869,15 +3883,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U21" s="9" t="inlineStr">
+      <c r="V21" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V21" t="n">
+      <c r="W21" t="n">
         <v>865</v>
       </c>
-      <c r="W21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -3954,15 +3968,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U22" s="9" t="inlineStr">
+      <c r="V22" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V22" t="n">
+      <c r="W22" t="n">
         <v>880</v>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4044,15 +4058,15 @@
           <t>K-0001</t>
         </is>
       </c>
-      <c r="U23" s="9" t="inlineStr">
+      <c r="V23" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V23" t="n">
+      <c r="W23" t="n">
         <v>895</v>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4134,15 +4148,15 @@
           <t>HK.03.01/1.3/395</t>
         </is>
       </c>
-      <c r="U24" s="9" t="inlineStr">
+      <c r="V24" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V24" t="n">
+      <c r="W24" t="n">
         <v>945</v>
       </c>
-      <c r="W24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4219,15 +4233,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U25" s="9" t="inlineStr">
+      <c r="V25" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V25" t="n">
+      <c r="W25" t="n">
         <v>960</v>
       </c>
-      <c r="W25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4309,15 +4323,15 @@
           <t>K-0010</t>
         </is>
       </c>
-      <c r="U26" s="9" t="inlineStr">
+      <c r="V26" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V26" t="n">
+      <c r="W26" t="n">
         <v>975</v>
       </c>
-      <c r="W26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4399,15 +4413,15 @@
           <t>K-0007</t>
         </is>
       </c>
-      <c r="U27" s="9" t="inlineStr">
+      <c r="V27" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V27" t="n">
+      <c r="W27" t="n">
         <v>995</v>
       </c>
-      <c r="W27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4484,15 +4498,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U28" s="9" t="inlineStr">
+      <c r="V28" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V28" t="n">
+      <c r="W28" t="n">
         <v>1015</v>
       </c>
-      <c r="W28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4569,15 +4583,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U29" s="9" t="inlineStr">
+      <c r="V29" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V29" t="n">
+      <c r="W29" t="n">
         <v>1035</v>
       </c>
-      <c r="W29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4654,15 +4668,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U30" s="9" t="inlineStr">
+      <c r="V30" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V30" t="n">
+      <c r="W30" t="n">
         <v>1100</v>
       </c>
-      <c r="W30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4739,15 +4753,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U31" s="9" t="inlineStr">
+      <c r="V31" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V31" t="n">
+      <c r="W31" t="n">
         <v>1125</v>
       </c>
-      <c r="W31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4824,15 +4838,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U32" s="9" t="inlineStr">
+      <c r="V32" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V32" t="n">
+      <c r="W32" t="n">
         <v>1225</v>
       </c>
-      <c r="W32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4909,15 +4923,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U33" s="9" t="inlineStr">
+      <c r="V33" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V33" t="n">
+      <c r="W33" t="n">
         <v>1315</v>
       </c>
-      <c r="W33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -4994,15 +5008,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U34" s="9" t="inlineStr">
+      <c r="V34" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V34" t="n">
+      <c r="W34" t="n">
         <v>1345</v>
       </c>
-      <c r="W34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5079,15 +5093,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U35" s="9" t="inlineStr">
+      <c r="V35" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V35" t="n">
+      <c r="W35" t="n">
         <v>1395</v>
       </c>
-      <c r="W35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5164,15 +5178,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U36" s="9" t="inlineStr">
+      <c r="V36" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V36" t="n">
+      <c r="W36" t="n">
         <v>1425</v>
       </c>
-      <c r="W36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5249,15 +5263,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U37" s="9" t="inlineStr">
+      <c r="V37" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V37" t="n">
+      <c r="W37" t="n">
         <v>1475</v>
       </c>
-      <c r="W37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5334,15 +5348,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U38" s="9" t="inlineStr">
+      <c r="V38" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V38" t="n">
+      <c r="W38" t="n">
         <v>1495</v>
       </c>
-      <c r="W38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5419,15 +5433,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U39" s="9" t="inlineStr">
+      <c r="V39" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V39" t="n">
+      <c r="W39" t="n">
         <v>1525</v>
       </c>
-      <c r="W39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5504,15 +5518,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U40" s="9" t="inlineStr">
+      <c r="V40" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V40" t="n">
+      <c r="W40" t="n">
         <v>1575</v>
       </c>
-      <c r="W40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5589,15 +5603,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U41" s="9" t="inlineStr">
+      <c r="V41" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V41" t="n">
+      <c r="W41" t="n">
         <v>1595</v>
       </c>
-      <c r="W41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5674,15 +5688,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U42" s="9" t="inlineStr">
+      <c r="V42" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V42" t="n">
+      <c r="W42" t="n">
         <v>1735</v>
       </c>
-      <c r="W42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5759,15 +5773,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U43" s="9" t="inlineStr">
+      <c r="V43" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V43" t="n">
+      <c r="W43" t="n">
         <v>1794</v>
       </c>
-      <c r="W43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5844,15 +5858,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U44" s="9" t="inlineStr">
+      <c r="V44" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V44" t="n">
+      <c r="W44" t="n">
         <v>2425</v>
       </c>
-      <c r="W44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -5929,15 +5943,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U45" s="9" t="inlineStr">
+      <c r="V45" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V45" t="n">
+      <c r="W45" t="n">
         <v>2725</v>
       </c>
-      <c r="W45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6014,15 +6028,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U46" s="9" t="inlineStr">
+      <c r="V46" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V46" t="n">
+      <c r="W46" t="n">
         <v>225</v>
       </c>
-      <c r="W46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6099,15 +6113,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U47" s="8" t="inlineStr">
+      <c r="V47" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V47" t="n">
+      <c r="W47" t="n">
         <v>-429</v>
       </c>
-      <c r="W47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6184,15 +6198,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U48" s="7" t="inlineStr">
+      <c r="V48" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V48" t="n">
+      <c r="W48" t="n">
         <v>11</v>
       </c>
-      <c r="W48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6274,15 +6288,15 @@
           <t>Menunggu konfirmasi mitra</t>
         </is>
       </c>
-      <c r="U49" s="9" t="inlineStr">
+      <c r="V49" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V49" t="n">
+      <c r="W49" t="n">
         <v>743</v>
       </c>
-      <c r="W49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6364,15 +6378,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U50" s="9" t="inlineStr">
+      <c r="V50" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V50" t="n">
+      <c r="W50" t="n">
         <v>1049</v>
       </c>
-      <c r="W50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6454,15 +6468,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U51" s="8" t="inlineStr">
+      <c r="V51" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V51" t="n">
+      <c r="W51" t="n">
         <v>-227</v>
       </c>
-      <c r="W51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6539,15 +6553,15 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="U52" s="8" t="inlineStr">
+      <c r="V52" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V52" t="n">
+      <c r="W52" t="n">
         <v>-420</v>
       </c>
-      <c r="W52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6624,15 +6638,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U53" s="7" t="inlineStr">
+      <c r="V53" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V53" t="n">
+      <c r="W53" t="n">
         <v>43</v>
       </c>
-      <c r="W53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6714,15 +6728,15 @@
           <t>Menunggu konfirmasi mitra</t>
         </is>
       </c>
-      <c r="U54" s="8" t="inlineStr">
+      <c r="V54" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V54" t="n">
+      <c r="W54" t="n">
         <v>-98</v>
       </c>
-      <c r="W54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6799,15 +6813,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U55" s="7" t="inlineStr">
+      <c r="V55" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V55" t="n">
+      <c r="W55" t="n">
         <v>35</v>
       </c>
-      <c r="W55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6889,15 +6903,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U56" s="8" t="inlineStr">
+      <c r="V56" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V56" t="n">
+      <c r="W56" t="n">
         <v>-154</v>
       </c>
-      <c r="W56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -6974,15 +6988,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U57" s="7" t="inlineStr">
+      <c r="V57" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V57" t="n">
+      <c r="W57" t="n">
         <v>23</v>
       </c>
-      <c r="W57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7064,15 +7078,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U58" s="7" t="inlineStr">
+      <c r="V58" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V58" t="n">
+      <c r="W58" t="n">
         <v>27</v>
       </c>
-      <c r="W58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7154,15 +7168,15 @@
           <t>Proses perpanjangan</t>
         </is>
       </c>
-      <c r="U59" s="9" t="inlineStr">
+      <c r="V59" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V59" t="n">
+      <c r="W59" t="n">
         <v>1185</v>
       </c>
-      <c r="W59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7239,15 +7253,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U60" s="7" t="inlineStr">
+      <c r="V60" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V60" t="n">
+      <c r="W60" t="n">
         <v>65</v>
       </c>
-      <c r="W60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7324,15 +7338,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U61" s="7" t="inlineStr">
+      <c r="V61" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V61" t="n">
+      <c r="W61" t="n">
         <v>18</v>
       </c>
-      <c r="W61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7414,15 +7428,15 @@
           <t>Menunggu konfirmasi mitra</t>
         </is>
       </c>
-      <c r="U62" s="9" t="inlineStr">
+      <c r="V62" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V62" t="n">
+      <c r="W62" t="n">
         <v>182</v>
       </c>
-      <c r="W62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7499,15 +7513,15 @@
           <t>Perpanjangan</t>
         </is>
       </c>
-      <c r="U63" s="9" t="inlineStr">
+      <c r="V63" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V63" t="n">
+      <c r="W63" t="n">
         <v>875</v>
       </c>
-      <c r="W63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7584,15 +7598,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U64" s="8" t="inlineStr">
+      <c r="V64" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V64" t="n">
+      <c r="W64" t="n">
         <v>-55</v>
       </c>
-      <c r="W64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7674,15 +7688,15 @@
           <t>Menunggu konfirmasi mitra</t>
         </is>
       </c>
-      <c r="U65" s="7" t="inlineStr">
+      <c r="V65" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V65" t="n">
+      <c r="W65" t="n">
         <v>6</v>
       </c>
-      <c r="W65" t="inlineStr">
+      <c r="X65" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7764,15 +7778,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U66" s="9" t="inlineStr">
+      <c r="V66" s="9" t="inlineStr">
         <is>
           <t>Aktif</t>
         </is>
       </c>
-      <c r="V66" t="n">
+      <c r="W66" t="n">
         <v>664</v>
       </c>
-      <c r="W66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7849,15 +7863,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U67" s="7" t="inlineStr">
+      <c r="V67" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V67" t="n">
+      <c r="W67" t="n">
         <v>28</v>
       </c>
-      <c r="W67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -7939,15 +7953,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U68" s="8" t="inlineStr">
+      <c r="V68" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V68" t="n">
+      <c r="W68" t="n">
         <v>-26</v>
       </c>
-      <c r="W68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8024,15 +8038,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U69" s="8" t="inlineStr">
+      <c r="V69" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V69" t="n">
+      <c r="W69" t="n">
         <v>-517</v>
       </c>
-      <c r="W69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8114,15 +8128,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U70" s="7" t="inlineStr">
+      <c r="V70" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V70" t="n">
+      <c r="W70" t="n">
         <v>47</v>
       </c>
-      <c r="W70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8204,15 +8218,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U71" s="8" t="inlineStr">
+      <c r="V71" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V71" t="n">
+      <c r="W71" t="n">
         <v>-73</v>
       </c>
-      <c r="W71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8289,15 +8303,15 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U72" s="8" t="inlineStr">
+      <c r="V72" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V72" t="n">
+      <c r="W72" t="n">
         <v>-214</v>
       </c>
-      <c r="W72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8379,15 +8393,15 @@
           <t>Perlu addendum</t>
         </is>
       </c>
-      <c r="U73" s="7" t="inlineStr">
+      <c r="V73" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V73" t="n">
+      <c r="W73" t="n">
         <v>23</v>
       </c>
-      <c r="W73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8469,15 +8483,15 @@
           <t>Proses perpanjangan</t>
         </is>
       </c>
-      <c r="U74" s="7" t="inlineStr">
+      <c r="V74" s="7" t="inlineStr">
         <is>
           <t>Segera Berakhir</t>
         </is>
       </c>
-      <c r="V74" t="n">
+      <c r="W74" t="n">
         <v>74</v>
       </c>
-      <c r="W74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8559,15 +8573,15 @@
           <t>Menunggu konfirmasi mitra</t>
         </is>
       </c>
-      <c r="U75" s="8" t="inlineStr">
+      <c r="V75" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V75" t="n">
+      <c r="W75" t="n">
         <v>-26</v>
       </c>
-      <c r="W75" t="inlineStr">
+      <c r="X75" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -8644,22 +8658,1686 @@
           <t>Baru</t>
         </is>
       </c>
-      <c r="U76" s="8" t="inlineStr">
+      <c r="V76" s="8" t="inlineStr">
         <is>
           <t>Habis</t>
         </is>
       </c>
-      <c r="V76" t="n">
+      <c r="W76" t="n">
         <v>-43</v>
       </c>
-      <c r="W76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>K-UJI-001</t>
+        </is>
+      </c>
+      <c r="B77" s="15" t="n">
+        <v>46224.99988977212</v>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>UJI COBA 01 — H-88</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>UJI/001</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" t="n">
+        <v>1</v>
+      </c>
+      <c r="N77" s="15" t="n">
+        <v>45943</v>
+      </c>
+      <c r="O77" s="15" t="n">
+        <v>46308</v>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr"/>
+      <c r="V77" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W77" t="n">
+        <v>88</v>
+      </c>
+      <c r="X77" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>K-UJI-002</t>
+        </is>
+      </c>
+      <c r="B78" s="15" t="n">
+        <v>46224.99988977237</v>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>UJI COBA 02 — H-75</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>UJI/002</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" t="n">
+        <v>1</v>
+      </c>
+      <c r="N78" s="15" t="n">
+        <v>45930</v>
+      </c>
+      <c r="O78" s="15" t="n">
+        <v>46295</v>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W78" t="n">
+        <v>75</v>
+      </c>
+      <c r="X78" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>K-UJI-003</t>
+        </is>
+      </c>
+      <c r="B79" s="15" t="n">
+        <v>46224.99988977248</v>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>UJI COBA 03 — H-66</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>UJI/003</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" t="n">
+        <v>1</v>
+      </c>
+      <c r="N79" s="15" t="n">
+        <v>45921</v>
+      </c>
+      <c r="O79" s="15" t="n">
+        <v>46286</v>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr"/>
+      <c r="V79" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W79" t="n">
+        <v>66</v>
+      </c>
+      <c r="X79" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>K-UJI-004</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="n">
+        <v>46224.99988977255</v>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>UJI COBA 04 — H-58</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>UJI/004</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" t="n">
+        <v>1</v>
+      </c>
+      <c r="N80" s="15" t="n">
+        <v>45913</v>
+      </c>
+      <c r="O80" s="15" t="n">
+        <v>46278</v>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr"/>
+      <c r="R80" t="inlineStr"/>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr"/>
+      <c r="V80" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W80" t="n">
+        <v>58</v>
+      </c>
+      <c r="X80" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>K-UJI-005</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="n">
+        <v>46224.99988977262</v>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>UJI COBA 05 — H-45</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>UJI/005</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" t="n">
+        <v>1</v>
+      </c>
+      <c r="N81" s="15" t="n">
+        <v>45900</v>
+      </c>
+      <c r="O81" s="15" t="n">
+        <v>46265</v>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr"/>
+      <c r="R81" t="inlineStr"/>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Tidak Diperpanjang</t>
+        </is>
+      </c>
+      <c r="V81" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W81" t="n">
+        <v>45</v>
+      </c>
+      <c r="X81" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>K-UJI-006</t>
+        </is>
+      </c>
+      <c r="B82" s="15" t="n">
+        <v>46224.99988977268</v>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>UJI COBA 06 — H-33</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>UJI/006</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" t="n">
+        <v>1</v>
+      </c>
+      <c r="N82" s="15" t="n">
+        <v>45888</v>
+      </c>
+      <c r="O82" s="15" t="n">
+        <v>46253</v>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr"/>
+      <c r="V82" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W82" t="n">
+        <v>33</v>
+      </c>
+      <c r="X82" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>K-UJI-007</t>
+        </is>
+      </c>
+      <c r="B83" s="15" t="n">
+        <v>46224.99988977274</v>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>UJI COBA 07 — H-28</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>UJI/007</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" t="n">
+        <v>1</v>
+      </c>
+      <c r="N83" s="15" t="n">
+        <v>45883</v>
+      </c>
+      <c r="O83" s="15" t="n">
+        <v>46248</v>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr"/>
+      <c r="V83" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W83" t="n">
+        <v>28</v>
+      </c>
+      <c r="X83" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>K-UJI-008</t>
+        </is>
+      </c>
+      <c r="B84" s="15" t="n">
+        <v>46224.99988977281</v>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>UJI COBA 08 — H-20</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>UJI/008</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" t="n">
+        <v>1</v>
+      </c>
+      <c r="N84" s="15" t="n">
+        <v>45875</v>
+      </c>
+      <c r="O84" s="15" t="n">
+        <v>46240</v>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr"/>
+      <c r="R84" t="inlineStr"/>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr"/>
+      <c r="V84" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W84" t="n">
+        <v>20</v>
+      </c>
+      <c r="X84" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>K-UJI-009</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="n">
+        <v>46224.99988977287</v>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>UJI COBA 09 — H-12</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>UJI/009</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr"/>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" t="n">
+        <v>1</v>
+      </c>
+      <c r="N85" s="15" t="n">
+        <v>45867</v>
+      </c>
+      <c r="O85" s="15" t="n">
+        <v>46232</v>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr"/>
+      <c r="R85" t="inlineStr"/>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr"/>
+      <c r="V85" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W85" t="n">
+        <v>12</v>
+      </c>
+      <c r="X85" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>K-UJI-010</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="n">
+        <v>46224.99988977293</v>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>UJI COBA 10 — H-9</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>UJI/010</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr"/>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
+      <c r="M86" t="n">
+        <v>1</v>
+      </c>
+      <c r="N86" s="15" t="n">
+        <v>45864</v>
+      </c>
+      <c r="O86" s="15" t="n">
+        <v>46229</v>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="inlineStr"/>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr"/>
+      <c r="V86" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W86" t="n">
+        <v>9</v>
+      </c>
+      <c r="X86" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>K-UJI-011</t>
+        </is>
+      </c>
+      <c r="B87" s="15" t="n">
+        <v>46224.999889773</v>
+      </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>UJI COBA 11 — H-7</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>UJI/011</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr"/>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
+      <c r="M87" t="n">
+        <v>1</v>
+      </c>
+      <c r="N87" s="15" t="n">
+        <v>45862</v>
+      </c>
+      <c r="O87" s="15" t="n">
+        <v>46227</v>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr"/>
+      <c r="R87" t="inlineStr"/>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr"/>
+      <c r="V87" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W87" t="n">
+        <v>7</v>
+      </c>
+      <c r="X87" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>K-UJI-012</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="n">
+        <v>46224.99988977305</v>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>UJI COBA 12 — H-5</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>UJI/012</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr"/>
+      <c r="L88" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" t="n">
+        <v>1</v>
+      </c>
+      <c r="N88" s="15" t="n">
+        <v>45860</v>
+      </c>
+      <c r="O88" s="15" t="n">
+        <v>46225</v>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr"/>
+      <c r="R88" t="inlineStr"/>
+      <c r="S88" t="inlineStr"/>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr"/>
+      <c r="V88" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W88" t="n">
+        <v>5</v>
+      </c>
+      <c r="X88" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>K-UJI-013</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="n">
+        <v>46224.99988977313</v>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>UJI COBA 13 — H-3</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>UJI/013</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr"/>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" t="n">
+        <v>1</v>
+      </c>
+      <c r="N89" s="15" t="n">
+        <v>45858</v>
+      </c>
+      <c r="O89" s="15" t="n">
+        <v>46223</v>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr"/>
+      <c r="R89" t="inlineStr"/>
+      <c r="S89" t="inlineStr"/>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr"/>
+      <c r="V89" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W89" t="n">
+        <v>3</v>
+      </c>
+      <c r="X89" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>K-UJI-014</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="n">
+        <v>46224.99988977319</v>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>UJI COBA 14 — H-1</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>UJI/014</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" t="n">
+        <v>1</v>
+      </c>
+      <c r="N90" s="15" t="n">
+        <v>45856</v>
+      </c>
+      <c r="O90" s="15" t="n">
+        <v>46221</v>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr"/>
+      <c r="R90" t="inlineStr"/>
+      <c r="S90" t="inlineStr"/>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr"/>
+      <c r="V90" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W90" t="n">
+        <v>1</v>
+      </c>
+      <c r="X90" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>K-UJI-015</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="n">
+        <v>46224.99988977325</v>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>UJI COBA 15 — HARI-H</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>UJI/015</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" t="n">
+        <v>1</v>
+      </c>
+      <c r="N91" s="15" t="n">
+        <v>45855</v>
+      </c>
+      <c r="O91" s="15" t="n">
+        <v>46220</v>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr"/>
+      <c r="R91" t="inlineStr"/>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr"/>
+      <c r="V91" s="7" t="inlineStr">
+        <is>
+          <t>Segera Berakhir</t>
+        </is>
+      </c>
+      <c r="W91" t="n">
+        <v>0</v>
+      </c>
+      <c r="X91" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>K-UJI-016</t>
+        </is>
+      </c>
+      <c r="B92" s="15" t="n">
+        <v>46224.99988977333</v>
+      </c>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>UJI COBA 16 — habis 1h</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>UJI/016</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" t="n">
+        <v>1</v>
+      </c>
+      <c r="N92" s="15" t="n">
+        <v>45854</v>
+      </c>
+      <c r="O92" s="15" t="n">
+        <v>46219</v>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr"/>
+      <c r="R92" t="inlineStr"/>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr"/>
+      <c r="V92" s="8" t="inlineStr">
+        <is>
+          <t>Habis</t>
+        </is>
+      </c>
+      <c r="W92" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X92" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>K-UJI-017</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="n">
+        <v>46224.99988977339</v>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>UJI COBA 17 — habis 3h</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>UJI/017</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="n">
+        <v>0</v>
+      </c>
+      <c r="M93" t="n">
+        <v>1</v>
+      </c>
+      <c r="N93" s="15" t="n">
+        <v>45852</v>
+      </c>
+      <c r="O93" s="15" t="n">
+        <v>46217</v>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr"/>
+      <c r="R93" t="inlineStr"/>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr"/>
+      <c r="V93" s="8" t="inlineStr">
+        <is>
+          <t>Habis</t>
+        </is>
+      </c>
+      <c r="W93" t="n">
+        <v>-3</v>
+      </c>
+      <c r="X93" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>K-UJI-018</t>
+        </is>
+      </c>
+      <c r="B94" s="15" t="n">
+        <v>46224.99988977346</v>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>UJI COBA 18 — habis 7h</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>UJI/018</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="n">
+        <v>0</v>
+      </c>
+      <c r="M94" t="n">
+        <v>1</v>
+      </c>
+      <c r="N94" s="15" t="n">
+        <v>45848</v>
+      </c>
+      <c r="O94" s="15" t="n">
+        <v>46213</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q94" t="inlineStr"/>
+      <c r="R94" t="inlineStr"/>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr"/>
+      <c r="V94" s="8" t="inlineStr">
+        <is>
+          <t>Habis</t>
+        </is>
+      </c>
+      <c r="W94" t="n">
+        <v>-7</v>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>K-UJI-019</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="n">
+        <v>46224.99988977353</v>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>UJI COBA 19 — habis 12h</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>UJI/019</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="n">
+        <v>0</v>
+      </c>
+      <c r="M95" t="n">
+        <v>1</v>
+      </c>
+      <c r="N95" s="15" t="n">
+        <v>45843</v>
+      </c>
+      <c r="O95" s="15" t="n">
+        <v>46208</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q95" t="inlineStr"/>
+      <c r="R95" t="inlineStr"/>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr"/>
+      <c r="V95" s="8" t="inlineStr">
+        <is>
+          <t>Habis</t>
+        </is>
+      </c>
+      <c r="W95" t="n">
+        <v>-12</v>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>K-UJI-020</t>
+        </is>
+      </c>
+      <c r="B96" s="15" t="n">
+        <v>46224.9998897736</v>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>UJI COBA 20 — habis 20h</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Uji Coba</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>UJI/020</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Perjanjian Kerja sama (PKS)</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Pendidikan</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Prodi DIII Gizi</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="n">
+        <v>0</v>
+      </c>
+      <c r="M96" t="n">
+        <v>1</v>
+      </c>
+      <c r="N96" s="15" t="n">
+        <v>45835</v>
+      </c>
+      <c r="O96" s="15" t="n">
+        <v>46200</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="Q96" t="inlineStr"/>
+      <c r="R96" t="inlineStr"/>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Data uji notif — boleh dihapus</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr"/>
+      <c r="V96" s="8" t="inlineStr">
+        <is>
+          <t>Habis</t>
+        </is>
+      </c>
+      <c r="W96" t="n">
+        <v>-20</v>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>uji@contoh.id</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:X76"/>
+  <autoFilter ref="A1:Y96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9365,12 +11043,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>NAMA_INSTANSI</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Politeknik Kesehatan Kemenkes Palembang</t>
         </is>
@@ -9382,12 +11060,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>EMAIL_NOTIF</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>kerjasama@poltekkespalembang.ac.id</t>
         </is>
@@ -9399,12 +11077,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>BASE_URL</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>https://simkerma.vercel.app</t>
         </is>
@@ -9416,12 +11094,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>REMINDER_CADENCE</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>90:30,60:14,30:7,7:1</t>
         </is>
@@ -9433,12 +11111,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>GRACE_HABIS_HARI</t>
         </is>
       </c>
-      <c r="B6" s="14" t="n">
+      <c r="B6" s="17" t="n">
         <v>14</v>
       </c>
       <c r="C6" s="12" t="inlineStr">
@@ -9448,12 +11126,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>EMAIL_AKTIF</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -9465,12 +11143,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>WA_NOMOR_AKTIF</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9482,12 +11160,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>WA_TARGET</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr"/>
+      <c r="B9" s="17" t="inlineStr"/>
       <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Nomor WA tim internal (mis. 62812xxxx), pisahkan koma</t>
@@ -9495,12 +11173,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>WA_GRUP_AKTIF</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9512,12 +11190,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>WA_GRUP_ID</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
+      <c r="B11" s="17" t="inlineStr"/>
       <c r="C11" s="12" t="inlineStr">
         <is>
           <t>ID grup WhatsApp (Fonnte) untuk rekap internal</t>
@@ -9525,12 +11203,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>LAMPIRKAN_FILE</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -9542,12 +11220,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>EMAIL_EKSTERNAL_AKTIF</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9559,12 +11237,12 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>WA_EKSTERNAL_AKTIF</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -9576,12 +11254,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>WA_EKSTERNAL_MAKS_PER_HARI</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="17" t="n">
         <v>8</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -9591,12 +11269,12 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>WA_EKSTERNAL_JEDA_DETIK</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
+      <c r="B16" s="17" t="n">
         <v>8</v>
       </c>
       <c r="C16" s="12" t="inlineStr">
@@ -9606,12 +11284,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>SURVEY_AKTIF</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>

</xml_diff>